<commit_message>
feat(design): Design B v2 — retours JLC integres
- Bandeau : chips SYSTEME et PROJET en evidence (aussi gros que le nom UO),
  badge SANTE a droite — bandeau identique sur toutes les feuilles
- Dashboard reorganise : cartes KPI -> rangee de 4 camemberts-jauges
  (avancement, heures, livrables, donnees d'entree) -> prochains livrables
  -> la balle est chez -> avancement des activites EN COURS uniquement
  (les terminees sont masquees, avec data bars)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projet_TrainSystem/Design_B_Cockpit.xlsx
+++ b/projet_TrainSystem/Design_B_Cockpit.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,12 @@
       <name val="Segoe UI"/>
       <color rgb="00B5D4F4"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -130,12 +136,18 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="005F5E5A"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -145,6 +157,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000C447C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00185FA5"/>
       </patternFill>
     </fill>
     <fill>
@@ -579,74 +596,76 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -654,16 +673,31 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -832,7 +866,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Avancement</a:t>
+              <a:t>Avancement — 45 %</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -864,18 +898,13 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="E6F1FB"/>
+                <a:srgbClr val="EFEDE7"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </dPt>
-          <cat>
-            <numRef>
-              <f>'_chart_data'!$A$1:$A$2</f>
-            </numRef>
-          </cat>
           <val>
             <numRef>
               <f>'_chart_data'!$B$1:$B$2</f>
@@ -883,7 +912,208 @@
           </val>
         </ser>
         <firstSliceAng val="0"/>
-        <holeSize val="62"/>
+        <holeSize val="60"/>
+      </doughnutChart>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Heures — 30 %</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <doughnutChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="888780"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="EFEDE7"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <val>
+            <numRef>
+              <f>'_chart_data'!$B$4:$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+        <holeSize val="60"/>
+      </doughnutChart>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Livrables — 33 %</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <doughnutChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="639922"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="EFEDE7"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <val>
+            <numRef>
+              <f>'_chart_data'!$B$7:$B$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+        <holeSize val="60"/>
+      </doughnutChart>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Données d'entrée — 67 %</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <doughnutChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="EF9F27"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="EFEDE7"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <val>
+            <numRef>
+              <f>'_chart_data'!$B$10:$B$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+        <holeSize val="60"/>
       </doughnutChart>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -898,10 +1128,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2376000" cy="2232000"/>
+    <ext cx="1655999" cy="1655999"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -911,6 +1141,72 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1655999" cy="1655999"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1655999" cy="1655999"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1655999" cy="1655999"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1209,7 +1505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1246,47 +1542,49 @@
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="3" t="inlineStr">
-        <is>
-          <t>SANTÉ ROUGE</t>
-        </is>
-      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Cockpit de pilotage · J. Dujardin</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
       <c r="P1" s="1" t="n"/>
       <c r="Q1" s="1" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Cockpit de pilotage   ·   Projet Demo · Climatisation · J. Dujardin</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
+          <t>⚙  SYSTÈME : CLIMATISATION</t>
+        </is>
+      </c>
       <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
-      <c r="L2" s="1" t="n"/>
-      <c r="P2" s="1" t="n"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>▣  PROJET : PROJET DEMO</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>SANTÉ ROUGE</t>
+        </is>
+      </c>
       <c r="Q2" s="1" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="5">
+      <c r="B3" s="6">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="6">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="6">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
@@ -1296,233 +1594,406 @@
       <c r="K3" s="1" t="n"/>
       <c r="L3" s="1" t="n"/>
       <c r="M3" s="1" t="n"/>
-      <c r="N3" s="1" t="n"/>
-      <c r="O3" s="1" t="n"/>
-      <c r="P3" s="1" t="n"/>
       <c r="Q3" s="1" t="n"/>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="12" t="n"/>
-      <c r="I5" s="13" t="n"/>
-      <c r="J5" s="14" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="10" t="n"/>
-      <c r="M5" s="11" t="n"/>
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="1" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="1" t="n"/>
+      <c r="O4" s="1" t="n"/>
+      <c r="P4" s="1" t="n"/>
+      <c r="Q4" s="1" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="12" t="n"/>
+      <c r="H6" s="13" t="n"/>
+      <c r="I6" s="14" t="n"/>
+      <c r="J6" s="15" t="n"/>
+      <c r="K6" s="10" t="n"/>
+      <c r="L6" s="11" t="n"/>
+      <c r="M6" s="12" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>AVANCEMENT UO</t>
         </is>
       </c>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>CONSOMMÉ</t>
         </is>
       </c>
-      <c r="G6" s="18" t="n"/>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="20" t="inlineStr">
         <is>
           <t>POINTS OUVERTS</t>
         </is>
       </c>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="17" t="inlineStr">
+      <c r="J7" s="21" t="n"/>
+      <c r="K7" s="18" t="inlineStr">
         <is>
           <t>EAC</t>
         </is>
       </c>
-      <c r="M6" s="18" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="B7" s="21" t="inlineStr">
+      <c r="M7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>45,0 %</t>
         </is>
       </c>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="22" t="inlineStr">
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="23" t="inlineStr">
         <is>
           <t>29,5 %</t>
         </is>
       </c>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="23" t="inlineStr">
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="24" t="inlineStr">
         <is>
           <t>2  ▲1</t>
         </is>
       </c>
-      <c r="J7" s="20" t="n"/>
-      <c r="K7" s="24" t="inlineStr">
+      <c r="J8" s="21" t="n"/>
+      <c r="K8" s="25" t="inlineStr">
         <is>
           <t>169 h</t>
         </is>
       </c>
-      <c r="M7" s="18" t="n"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="B8" s="25" t="inlineStr">
+      <c r="M8" s="19" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>pondéré par poids</t>
         </is>
       </c>
-      <c r="C8" s="26" t="n"/>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="C9" s="27" t="n"/>
+      <c r="D9" s="28" t="n"/>
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>59 h / 200 h</t>
         </is>
       </c>
-      <c r="F8" s="29" t="n"/>
-      <c r="G8" s="30" t="n"/>
-      <c r="H8" s="31" t="inlineStr">
+      <c r="F9" s="30" t="n"/>
+      <c r="G9" s="31" t="n"/>
+      <c r="H9" s="32" t="inlineStr">
         <is>
           <t>dont 1 critique</t>
         </is>
       </c>
-      <c r="I8" s="32" t="n"/>
-      <c r="J8" s="33" t="n"/>
-      <c r="K8" s="28" t="inlineStr">
+      <c r="I9" s="33" t="n"/>
+      <c r="J9" s="34" t="n"/>
+      <c r="K9" s="29" t="inlineStr">
         <is>
           <t>dérive −31 h</t>
         </is>
       </c>
-      <c r="L8" s="29" t="n"/>
-      <c r="M8" s="30" t="n"/>
-    </row>
-    <row r="10">
-      <c r="F10" s="34" t="inlineStr">
+      <c r="L9" s="30" t="n"/>
+      <c r="M9" s="31" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>Prochains livrables</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
-      <c r="F11" s="35" t="inlineStr">
+    <row r="22" ht="19" customHeight="1">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t>SAA.RS — Requirement Spec</t>
         </is>
       </c>
-      <c r="G11" s="36" t="n"/>
-      <c r="H11" s="36" t="n"/>
-      <c r="I11" s="36" t="n"/>
-      <c r="J11" s="36" t="n"/>
-      <c r="K11" s="37" t="inlineStr">
+      <c r="C22" s="37" t="n"/>
+      <c r="D22" s="37" t="n"/>
+      <c r="E22" s="37" t="n"/>
+      <c r="F22" s="37" t="n"/>
+      <c r="G22" s="37" t="n"/>
+      <c r="H22" s="37" t="n"/>
+      <c r="I22" s="38" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="L11" s="38" t="inlineStr">
+      <c r="J22" s="39" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="M11" s="36" t="n"/>
-    </row>
-    <row r="12" ht="19" customHeight="1">
-      <c r="F12" s="35" t="inlineStr">
+      <c r="K22" s="37" t="n"/>
+    </row>
+    <row r="23" ht="19" customHeight="1">
+      <c r="B23" s="36" t="inlineStr">
         <is>
           <t>RSS.RS — Subsystem Spec</t>
         </is>
       </c>
-      <c r="G12" s="36" t="n"/>
-      <c r="H12" s="36" t="n"/>
-      <c r="I12" s="36" t="n"/>
-      <c r="J12" s="36" t="n"/>
-      <c r="K12" s="37" t="inlineStr">
+      <c r="C23" s="37" t="n"/>
+      <c r="D23" s="37" t="n"/>
+      <c r="E23" s="37" t="n"/>
+      <c r="F23" s="37" t="n"/>
+      <c r="G23" s="37" t="n"/>
+      <c r="H23" s="37" t="n"/>
+      <c r="I23" s="38" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="L12" s="38" t="inlineStr">
+      <c r="J23" s="39" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="M12" s="36" t="n"/>
-    </row>
-    <row r="13" ht="19" customHeight="1">
-      <c r="F13" s="35" t="inlineStr">
+      <c r="K23" s="37" t="n"/>
+    </row>
+    <row r="24" ht="19" customHeight="1">
+      <c r="B24" s="36" t="inlineStr">
         <is>
           <t>DR.RS — Design Review file</t>
         </is>
       </c>
-      <c r="G13" s="36" t="n"/>
-      <c r="H13" s="36" t="n"/>
-      <c r="I13" s="36" t="n"/>
-      <c r="J13" s="36" t="n"/>
-      <c r="K13" s="37" t="inlineStr">
+      <c r="C24" s="37" t="n"/>
+      <c r="D24" s="37" t="n"/>
+      <c r="E24" s="37" t="n"/>
+      <c r="F24" s="37" t="n"/>
+      <c r="G24" s="37" t="n"/>
+      <c r="H24" s="37" t="n"/>
+      <c r="I24" s="38" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L13" s="38" t="inlineStr">
+      <c r="J24" s="39" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="M13" s="36" t="n"/>
-    </row>
-    <row r="15">
-      <c r="F15" s="34" t="inlineStr">
+      <c r="K24" s="37" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>La balle est chez…</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="F16" s="39" t="inlineStr">
+    <row r="27" ht="22" customHeight="1">
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>FOURNISSEUR : 1</t>
         </is>
       </c>
-      <c r="I16" s="40" t="inlineStr">
+      <c r="E27" s="41" t="inlineStr">
         <is>
           <t>EXPERT : 1</t>
         </is>
       </c>
-      <c r="L16" s="41" t="inlineStr">
+      <c r="H27" s="42" t="inlineStr">
         <is>
           <t>NOUS (SE) : 0</t>
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>Avancement des activités en cours</t>
+        </is>
+      </c>
+      <c r="I29" s="43" t="inlineStr">
+        <is>
+          <t>(les activités terminées ne sont pas affichées)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>activité</t>
+        </is>
+      </c>
+      <c r="C30" s="37" t="n"/>
+      <c r="D30" s="37" t="n"/>
+      <c r="E30" s="37" t="n"/>
+      <c r="F30" s="37" t="n"/>
+      <c r="G30" s="37" t="n"/>
+      <c r="H30" s="37" t="n"/>
+      <c r="I30" s="44" t="inlineStr">
+        <is>
+          <t>statut</t>
+        </is>
+      </c>
+      <c r="J30" s="37" t="n"/>
+      <c r="K30" s="44" t="inlineStr">
+        <is>
+          <t>avancement</t>
+        </is>
+      </c>
+      <c r="L30" s="37" t="n"/>
+      <c r="M30" s="37" t="n"/>
+      <c r="N30" s="44" t="inlineStr">
+        <is>
+          <t>heures</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="19" customHeight="1">
+      <c r="B31" s="45" t="inlineStr">
+        <is>
+          <t>ACT-02 — Specification des exigences</t>
+        </is>
+      </c>
+      <c r="I31" s="46" t="inlineStr">
+        <is>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="K31" s="46" t="n">
+        <v>60</v>
+      </c>
+      <c r="N31" s="47" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="32" ht="19" customHeight="1">
+      <c r="B32" s="45" t="inlineStr">
+        <is>
+          <t>ACT-03 — Definition d'architecture</t>
+        </is>
+      </c>
+      <c r="I32" s="46" t="inlineStr">
+        <is>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="K32" s="46" t="n">
+        <v>35</v>
+      </c>
+      <c r="N32" s="47" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" ht="19" customHeight="1">
+      <c r="B33" s="45" t="inlineStr">
+        <is>
+          <t>ACT-04 — Calculs et simulations</t>
+        </is>
+      </c>
+      <c r="I33" s="46" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="K33" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" ht="19" customHeight="1">
+      <c r="B34" s="45" t="inlineStr">
+        <is>
+          <t>ACT-05 — Revue de conception</t>
+        </is>
+      </c>
+      <c r="I34" s="46" t="inlineStr">
+        <is>
+          <t>A_FAIRE</t>
+        </is>
+      </c>
+      <c r="K34" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" ht="19" customHeight="1">
+      <c r="B35" s="45" t="inlineStr">
+        <is>
+          <t>ACT-06 — Preparation gate review</t>
+        </is>
+      </c>
+      <c r="I35" s="46" t="inlineStr">
+        <is>
+          <t>STAND_BY</t>
+        </is>
+      </c>
+      <c r="K35" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="N35" s="47" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="F11:J11"/>
-    <mergeCell ref="F16:G16"/>
+  <mergeCells count="43">
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="K32:M32"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="L16:M16"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="K31:M31"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="B33:H33"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="H7:J7"/>
-    <mergeCell ref="E6:G6"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="K8:M8"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="F12:J12"/>
-    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="B32:H32"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="B9:D9"/>
     <mergeCell ref="E7:G7"/>
-    <mergeCell ref="B6:D6"/>
     <mergeCell ref="K7:M7"/>
-    <mergeCell ref="M1:O2"/>
-    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="N2:P3"/>
+    <mergeCell ref="I33:J33"/>
     <mergeCell ref="H8:J8"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="K34:M34"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="K9:M9"/>
     <mergeCell ref="E8:G8"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="B34:H34"/>
   </mergeCells>
-  <conditionalFormatting sqref="L11:L13">
+  <conditionalFormatting sqref="J22:J24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"TERMINEE"</formula>
     </cfRule>
@@ -1533,6 +2004,29 @@
       <formula>"STAND_BY"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"A_FAIRE"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K31:K35">
+    <cfRule type="dataBar" priority="5">
+      <dataBar showValue="1">
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="00378ADD"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I31:I35">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
+      <formula>"TERMINEE"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="1">
+      <formula>"EN_COURS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="2">
+      <formula>"STAND_BY"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="3">
       <formula>"A_FAIRE"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1547,7 +2041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1568,6 +2062,66 @@
       </c>
       <c r="B2" t="n">
         <v>55</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fait</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>reste</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fait</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>reste</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fait</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>reste</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1582,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1609,38 +2163,37 @@
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="16" customHeight="1">
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Saisie — Activités · J. Dujardin</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Saisie — Activités   ·   Projet Demo · Climatisation · J. Dujardin</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
+          <t>⚙  SYSTÈME : CLIMATISATION</t>
+        </is>
+      </c>
       <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
-      <c r="L2" s="1" t="n"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>▣  PROJET : PROJET DEMO</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="5">
+      <c r="B3" s="6">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="6">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="6">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
@@ -1650,224 +2203,241 @@
       <c r="K3" s="1" t="n"/>
       <c r="L3" s="1" t="n"/>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="42" t="inlineStr">
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="1" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="48" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B6" s="48" t="inlineStr">
         <is>
           <t>designation</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C6" s="48" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D6" s="48" t="inlineStr">
         <is>
           <t>avancement</t>
         </is>
       </c>
-      <c r="E5" s="42" t="inlineStr">
+      <c r="E6" s="48" t="inlineStr">
         <is>
           <t>load (h)</t>
         </is>
       </c>
-      <c r="F5" s="42" t="inlineStr">
+      <c r="F6" s="48" t="inlineStr">
         <is>
           <t>consommé (h)</t>
         </is>
       </c>
-      <c r="G5" s="42" t="inlineStr">
+      <c r="G6" s="48" t="inlineStr">
         <is>
           <t>reste (h)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="43" t="inlineStr">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>ACT-01</t>
         </is>
       </c>
-      <c r="B6" s="44" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>Analyse fonctionnelle du besoin</t>
         </is>
       </c>
-      <c r="C6" s="43" t="inlineStr">
+      <c r="C7" s="49" t="inlineStr">
         <is>
           <t>TERMINEE</t>
         </is>
       </c>
-      <c r="D6" s="43" t="n">
+      <c r="D7" s="49" t="n">
         <v>100</v>
       </c>
-      <c r="E6" s="45" t="n">
+      <c r="E7" s="51" t="n">
         <v>24</v>
       </c>
-      <c r="F6" s="45" t="n">
+      <c r="F7" s="51" t="n">
         <v>22</v>
       </c>
-      <c r="G6" s="45" t="n">
+      <c r="G7" s="51" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>ACT-02</t>
         </is>
       </c>
-      <c r="B7" s="44" t="inlineStr">
+      <c r="B8" s="50" t="inlineStr">
         <is>
           <t>Specification des exigences</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="D7" s="43" t="n">
+      <c r="D8" s="49" t="n">
         <v>60</v>
       </c>
-      <c r="E7" s="45" t="n">
+      <c r="E8" s="51" t="n">
         <v>30</v>
       </c>
-      <c r="F7" s="45" t="n">
+      <c r="F8" s="51" t="n">
         <v>28.5</v>
       </c>
-      <c r="G7" s="45" t="n">
+      <c r="G8" s="51" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t>ACT-03</t>
         </is>
       </c>
-      <c r="B8" s="44" t="inlineStr">
+      <c r="B9" s="50" t="inlineStr">
         <is>
           <t>Definition d'architecture</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="D8" s="43" t="n">
+      <c r="D9" s="49" t="n">
         <v>35</v>
       </c>
-      <c r="E8" s="45" t="n">
+      <c r="E9" s="51" t="n">
         <v>40</v>
       </c>
-      <c r="F8" s="45" t="n">
+      <c r="F9" s="51" t="n">
         <v>12</v>
       </c>
-      <c r="G8" s="45" t="n">
+      <c r="G9" s="51" t="n">
         <v>26</v>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="43" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>ACT-04</t>
         </is>
       </c>
-      <c r="B9" s="44" t="inlineStr">
+      <c r="B10" s="50" t="inlineStr">
         <is>
           <t>Calculs et simulations</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="D9" s="43" t="n">
+      <c r="D10" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="45" t="n">
+      <c r="E10" s="51" t="n">
         <v>35</v>
       </c>
-      <c r="F9" s="45" t="n">
+      <c r="F10" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="45" t="n">
+      <c r="G10" s="51" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="43" t="inlineStr">
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="49" t="inlineStr">
         <is>
           <t>ACT-05</t>
         </is>
       </c>
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B11" s="50" t="inlineStr">
         <is>
           <t>Revue de conception</t>
         </is>
       </c>
-      <c r="C10" s="43" t="inlineStr">
+      <c r="C11" s="49" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="D10" s="43" t="n">
+      <c r="D11" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="45" t="n">
+      <c r="E11" s="51" t="n">
         <v>25</v>
       </c>
-      <c r="F10" s="45" t="n">
+      <c r="F11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="45" t="n">
+      <c r="G11" s="51" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="43" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t>ACT-06</t>
         </is>
       </c>
-      <c r="B11" s="44" t="inlineStr">
+      <c r="B12" s="50" t="inlineStr">
         <is>
           <t>Preparation gate review</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C12" s="49" t="inlineStr">
         <is>
           <t>STAND_BY</t>
         </is>
       </c>
-      <c r="D11" s="43" t="n">
+      <c r="D12" s="49" t="n">
         <v>10</v>
       </c>
-      <c r="E11" s="45" t="n">
+      <c r="E12" s="51" t="n">
         <v>46</v>
       </c>
-      <c r="F11" s="45" t="n">
+      <c r="F12" s="51" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="45" t="n">
+      <c r="G12" s="51" t="n">
         <v>41.4</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:C3"/>
+    <mergeCell ref="K1:L1"/>
     <mergeCell ref="D3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D11">
+  <conditionalFormatting sqref="D7:D12">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -1876,7 +2446,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C11">
+  <conditionalFormatting sqref="C7:C12">
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"TERMINEE"</formula>
     </cfRule>
@@ -1901,7 +2471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1926,34 +2496,37 @@
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="16" customHeight="1">
+      <c r="K1" s="52" t="inlineStr">
+        <is>
+          <t>Points ouverts — OIL · J. Dujardin</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Points ouverts — OIL   ·   Projet Demo · Climatisation · J. Dujardin</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
+          <t>⚙  SYSTÈME : CLIMATISATION</t>
+        </is>
+      </c>
       <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>▣  PROJET : PROJET DEMO</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="5">
+      <c r="B3" s="6">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="6">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="6">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
@@ -1961,121 +2534,136 @@
       <c r="I3" s="1" t="n"/>
       <c r="J3" s="1" t="n"/>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="42" t="inlineStr">
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="48" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B6" s="48" t="inlineStr">
         <is>
           <t>titre</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C6" s="48" t="inlineStr">
         <is>
           <t>en_action</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D6" s="48" t="inlineStr">
         <is>
           <t>criticite</t>
         </is>
       </c>
-      <c r="E5" s="42" t="inlineStr">
+      <c r="E6" s="48" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="43" t="inlineStr">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>PO-001</t>
         </is>
       </c>
-      <c r="B6" s="44" t="inlineStr">
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>Question expert normes EN 45545</t>
         </is>
       </c>
-      <c r="C6" s="43" t="inlineStr">
+      <c r="C7" s="49" t="inlineStr">
         <is>
           <t>EXPERT</t>
         </is>
       </c>
-      <c r="D6" s="43" t="inlineStr">
+      <c r="D7" s="49" t="inlineStr">
         <is>
           <t>HAUTE</t>
         </is>
       </c>
-      <c r="E6" s="43" t="inlineStr">
+      <c r="E7" s="49" t="inlineStr">
         <is>
           <t>OUVERT</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>PO-002</t>
         </is>
       </c>
-      <c r="B7" s="44" t="inlineStr">
+      <c r="B8" s="50" t="inlineStr">
         <is>
           <t>Attente retour relecture fournisseur</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>FOURNISSEUR</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
+      <c r="D8" s="49" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
-      <c r="E7" s="43" t="inlineStr">
+      <c r="E8" s="49" t="inlineStr">
         <is>
           <t>OUVERT</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t>PO-003</t>
         </is>
       </c>
-      <c r="B8" s="44" t="inlineStr">
+      <c r="B9" s="50" t="inlineStr">
         <is>
           <t>Acces outil documentaire obtenu</t>
         </is>
       </c>
-      <c r="C8" s="43" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
         <is>
           <t>SE</t>
         </is>
       </c>
-      <c r="D8" s="43" t="inlineStr">
+      <c r="D9" s="49" t="inlineStr">
         <is>
           <t>BASSE</t>
         </is>
       </c>
-      <c r="E8" s="43" t="inlineStr">
+      <c r="E9" s="49" t="inlineStr">
         <is>
           <t>CLOS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:C3"/>
+    <mergeCell ref="K1:L1"/>
     <mergeCell ref="D3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D8">
+  <conditionalFormatting sqref="D7:D9">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="4">
       <formula>"HAUTE"</formula>
     </cfRule>
@@ -2086,7 +2674,7 @@
       <formula>"BASSE"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E8">
+  <conditionalFormatting sqref="E7:E9">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="4">
       <formula>"OUVERT"</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat(design): Design B v3 — badge 1 ligne, chips epurees, bandeau colore par onglet, zones delimitees
- Badge SANTE sur une seule ligne du bandeau
- Chips : juste le nom (CLIMATISATION / PROJET DEMO), sans prefixe
- Couleur de bandeau = couleur d'onglet : Dashboard marine, Activites
  teal, OIL ambre — on sait ou on est d'un coup d'oeil
- Zones Livrables / Balle / Activites en cours : bande de titre remplie
  + cadre fin (section_box)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projet_TrainSystem/Design_B_Cockpit.xlsx
+++ b/projet_TrainSystem/Design_B_Cockpit.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -142,12 +142,34 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <color rgb="009FE1CB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="009FE1CB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00FAC775"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FAC775"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -176,6 +198,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E6F1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FAEEDA"/>
       </patternFill>
     </fill>
@@ -189,6 +216,26 @@
         <fgColor rgb="00EAF3DE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F6E56"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00085041"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BA7517"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00854F0B"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="43">
     <border>
@@ -596,7 +643,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -658,7 +705,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -667,25 +718,39 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -697,9 +762,15 @@
     <xf numFmtId="164" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1505,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1557,13 +1628,13 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>⚙  SYSTÈME : CLIMATISATION</t>
+          <t>⚙  CLIMATISATION</t>
         </is>
       </c>
       <c r="G2" s="1" t="n"/>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>▣  PROJET : PROJET DEMO</t>
+          <t>▣  PROJET DEMO</t>
         </is>
       </c>
       <c r="M2" s="1" t="n"/>
@@ -1594,6 +1665,9 @@
       <c r="K3" s="1" t="n"/>
       <c r="L3" s="1" t="n"/>
       <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
+      <c r="P3" s="1" t="n"/>
       <c r="Q3" s="1" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1">
@@ -1711,283 +1785,379 @@
       <c r="L9" s="30" t="n"/>
       <c r="M9" s="31" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="20" customHeight="1">
       <c r="B21" s="35" t="inlineStr">
         <is>
           <t>Prochains livrables</t>
         </is>
       </c>
+      <c r="C21" s="36" t="n"/>
+      <c r="D21" s="36" t="n"/>
+      <c r="E21" s="36" t="n"/>
+      <c r="F21" s="36" t="n"/>
+      <c r="G21" s="36" t="n"/>
+      <c r="H21" s="36" t="n"/>
+      <c r="I21" s="36" t="n"/>
+      <c r="J21" s="36" t="n"/>
+      <c r="K21" s="36" t="n"/>
+      <c r="L21" s="36" t="n"/>
+      <c r="M21" s="36" t="n"/>
+      <c r="N21" s="37" t="n"/>
     </row>
     <row r="22" ht="19" customHeight="1">
-      <c r="B22" s="36" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>SAA.RS — Requirement Spec</t>
         </is>
       </c>
-      <c r="C22" s="37" t="n"/>
-      <c r="D22" s="37" t="n"/>
-      <c r="E22" s="37" t="n"/>
-      <c r="F22" s="37" t="n"/>
-      <c r="G22" s="37" t="n"/>
-      <c r="H22" s="37" t="n"/>
-      <c r="I22" s="38" t="inlineStr">
+      <c r="C22" s="39" t="n"/>
+      <c r="D22" s="39" t="n"/>
+      <c r="E22" s="39" t="n"/>
+      <c r="F22" s="39" t="n"/>
+      <c r="G22" s="39" t="n"/>
+      <c r="H22" s="39" t="n"/>
+      <c r="I22" s="40" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="J22" s="39" t="inlineStr">
+      <c r="J22" s="41" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="K22" s="37" t="n"/>
+      <c r="K22" s="39" t="n"/>
+      <c r="L22" s="42" t="n"/>
+      <c r="M22" s="42" t="n"/>
+      <c r="N22" s="43" t="n"/>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="B23" s="36" t="inlineStr">
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>RSS.RS — Subsystem Spec</t>
         </is>
       </c>
-      <c r="C23" s="37" t="n"/>
-      <c r="D23" s="37" t="n"/>
-      <c r="E23" s="37" t="n"/>
-      <c r="F23" s="37" t="n"/>
-      <c r="G23" s="37" t="n"/>
-      <c r="H23" s="37" t="n"/>
-      <c r="I23" s="38" t="inlineStr">
+      <c r="C23" s="39" t="n"/>
+      <c r="D23" s="39" t="n"/>
+      <c r="E23" s="39" t="n"/>
+      <c r="F23" s="39" t="n"/>
+      <c r="G23" s="39" t="n"/>
+      <c r="H23" s="39" t="n"/>
+      <c r="I23" s="40" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="J23" s="39" t="inlineStr">
+      <c r="J23" s="41" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K23" s="37" t="n"/>
+      <c r="K23" s="39" t="n"/>
+      <c r="L23" s="42" t="n"/>
+      <c r="M23" s="42" t="n"/>
+      <c r="N23" s="43" t="n"/>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="B24" s="36" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>DR.RS — Design Review file</t>
         </is>
       </c>
-      <c r="C24" s="37" t="n"/>
-      <c r="D24" s="37" t="n"/>
-      <c r="E24" s="37" t="n"/>
-      <c r="F24" s="37" t="n"/>
-      <c r="G24" s="37" t="n"/>
-      <c r="H24" s="37" t="n"/>
-      <c r="I24" s="38" t="inlineStr">
+      <c r="C24" s="39" t="n"/>
+      <c r="D24" s="39" t="n"/>
+      <c r="E24" s="39" t="n"/>
+      <c r="F24" s="39" t="n"/>
+      <c r="G24" s="39" t="n"/>
+      <c r="H24" s="39" t="n"/>
+      <c r="I24" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J24" s="39" t="inlineStr">
+      <c r="J24" s="41" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K24" s="37" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="35" t="inlineStr">
+      <c r="K24" s="39" t="n"/>
+      <c r="L24" s="42" t="n"/>
+      <c r="M24" s="42" t="n"/>
+      <c r="N24" s="43" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="44" t="n"/>
+      <c r="C25" s="45" t="n"/>
+      <c r="D25" s="45" t="n"/>
+      <c r="E25" s="45" t="n"/>
+      <c r="F25" s="45" t="n"/>
+      <c r="G25" s="45" t="n"/>
+      <c r="H25" s="45" t="n"/>
+      <c r="I25" s="45" t="n"/>
+      <c r="J25" s="45" t="n"/>
+      <c r="K25" s="45" t="n"/>
+      <c r="L25" s="45" t="n"/>
+      <c r="M25" s="45" t="n"/>
+      <c r="N25" s="46" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>La balle est chez…</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="40" t="inlineStr">
+      <c r="C27" s="36" t="n"/>
+      <c r="D27" s="36" t="n"/>
+      <c r="E27" s="36" t="n"/>
+      <c r="F27" s="36" t="n"/>
+      <c r="G27" s="36" t="n"/>
+      <c r="H27" s="36" t="n"/>
+      <c r="I27" s="36" t="n"/>
+      <c r="J27" s="36" t="n"/>
+      <c r="K27" s="36" t="n"/>
+      <c r="L27" s="36" t="n"/>
+      <c r="M27" s="36" t="n"/>
+      <c r="N27" s="37" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="47" t="inlineStr">
         <is>
           <t>FOURNISSEUR : 1</t>
         </is>
       </c>
-      <c r="E27" s="41" t="inlineStr">
+      <c r="D28" s="42" t="n"/>
+      <c r="E28" s="48" t="inlineStr">
         <is>
           <t>EXPERT : 1</t>
         </is>
       </c>
-      <c r="H27" s="42" t="inlineStr">
+      <c r="G28" s="42" t="n"/>
+      <c r="H28" s="49" t="inlineStr">
         <is>
           <t>NOUS (SE) : 0</t>
         </is>
       </c>
+      <c r="J28" s="42" t="n"/>
+      <c r="K28" s="42" t="n"/>
+      <c r="L28" s="42" t="n"/>
+      <c r="M28" s="42" t="n"/>
+      <c r="N28" s="43" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="35" t="inlineStr">
+      <c r="B29" s="44" t="n"/>
+      <c r="C29" s="45" t="n"/>
+      <c r="D29" s="45" t="n"/>
+      <c r="E29" s="45" t="n"/>
+      <c r="F29" s="45" t="n"/>
+      <c r="G29" s="45" t="n"/>
+      <c r="H29" s="45" t="n"/>
+      <c r="I29" s="45" t="n"/>
+      <c r="J29" s="45" t="n"/>
+      <c r="K29" s="45" t="n"/>
+      <c r="L29" s="45" t="n"/>
+      <c r="M29" s="45" t="n"/>
+      <c r="N29" s="46" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="B31" s="35" t="inlineStr">
         <is>
           <t>Avancement des activités en cours</t>
         </is>
       </c>
-      <c r="I29" s="43" t="inlineStr">
+      <c r="C31" s="36" t="n"/>
+      <c r="D31" s="36" t="n"/>
+      <c r="E31" s="36" t="n"/>
+      <c r="F31" s="36" t="n"/>
+      <c r="G31" s="36" t="n"/>
+      <c r="H31" s="36" t="n"/>
+      <c r="I31" s="50" t="inlineStr">
         <is>
           <t>(les activités terminées ne sont pas affichées)</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="44" t="inlineStr">
+      <c r="J31" s="36" t="n"/>
+      <c r="K31" s="36" t="n"/>
+      <c r="L31" s="36" t="n"/>
+      <c r="M31" s="36" t="n"/>
+      <c r="N31" s="37" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="51" t="inlineStr">
         <is>
           <t>activité</t>
         </is>
       </c>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="37" t="n"/>
-      <c r="E30" s="37" t="n"/>
-      <c r="F30" s="37" t="n"/>
-      <c r="G30" s="37" t="n"/>
-      <c r="H30" s="37" t="n"/>
-      <c r="I30" s="44" t="inlineStr">
+      <c r="C32" s="39" t="n"/>
+      <c r="D32" s="39" t="n"/>
+      <c r="E32" s="39" t="n"/>
+      <c r="F32" s="39" t="n"/>
+      <c r="G32" s="39" t="n"/>
+      <c r="H32" s="39" t="n"/>
+      <c r="I32" s="51" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
-      <c r="J30" s="37" t="n"/>
-      <c r="K30" s="44" t="inlineStr">
+      <c r="J32" s="39" t="n"/>
+      <c r="K32" s="51" t="inlineStr">
         <is>
           <t>avancement</t>
         </is>
       </c>
-      <c r="L30" s="37" t="n"/>
-      <c r="M30" s="37" t="n"/>
-      <c r="N30" s="44" t="inlineStr">
+      <c r="L32" s="39" t="n"/>
+      <c r="M32" s="39" t="n"/>
+      <c r="N32" s="51" t="inlineStr">
         <is>
           <t>heures</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="B31" s="45" t="inlineStr">
+    <row r="33" ht="19" customHeight="1">
+      <c r="B33" s="52" t="inlineStr">
         <is>
           <t>ACT-02 — Specification des exigences</t>
         </is>
       </c>
-      <c r="I31" s="46" t="inlineStr">
+      <c r="I33" s="53" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="K31" s="46" t="n">
+      <c r="K33" s="53" t="n">
         <v>60</v>
       </c>
-      <c r="N31" s="47" t="n">
+      <c r="N33" s="54" t="n">
         <v>28.5</v>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
-      <c r="B32" s="45" t="inlineStr">
+    <row r="34" ht="19" customHeight="1">
+      <c r="B34" s="52" t="inlineStr">
         <is>
           <t>ACT-03 — Definition d'architecture</t>
         </is>
       </c>
-      <c r="I32" s="46" t="inlineStr">
+      <c r="I34" s="53" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="K32" s="46" t="n">
+      <c r="K34" s="53" t="n">
         <v>35</v>
       </c>
-      <c r="N32" s="47" t="n">
+      <c r="N34" s="54" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="B33" s="45" t="inlineStr">
+    <row r="35" ht="19" customHeight="1">
+      <c r="B35" s="52" t="inlineStr">
         <is>
           <t>ACT-04 — Calculs et simulations</t>
         </is>
       </c>
-      <c r="I33" s="46" t="inlineStr">
+      <c r="I35" s="53" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K33" s="46" t="n">
+      <c r="K35" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="N33" s="47" t="n">
+      <c r="N35" s="54" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="B34" s="45" t="inlineStr">
+    <row r="36" ht="19" customHeight="1">
+      <c r="B36" s="52" t="inlineStr">
         <is>
           <t>ACT-05 — Revue de conception</t>
         </is>
       </c>
-      <c r="I34" s="46" t="inlineStr">
+      <c r="I36" s="53" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K34" s="46" t="n">
+      <c r="K36" s="53" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="47" t="n">
+      <c r="N36" s="54" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="35" ht="19" customHeight="1">
-      <c r="B35" s="45" t="inlineStr">
+    <row r="37" ht="19" customHeight="1">
+      <c r="B37" s="52" t="inlineStr">
         <is>
           <t>ACT-06 — Preparation gate review</t>
         </is>
       </c>
-      <c r="I35" s="46" t="inlineStr">
+      <c r="I37" s="53" t="inlineStr">
         <is>
           <t>STAND_BY</t>
         </is>
       </c>
-      <c r="K35" s="46" t="n">
+      <c r="K37" s="53" t="n">
         <v>10</v>
       </c>
-      <c r="N35" s="47" t="n">
+      <c r="N37" s="54" t="n">
         <v>4</v>
       </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="44" t="n"/>
+      <c r="C38" s="45" t="n"/>
+      <c r="D38" s="45" t="n"/>
+      <c r="E38" s="45" t="n"/>
+      <c r="F38" s="45" t="n"/>
+      <c r="G38" s="45" t="n"/>
+      <c r="H38" s="45" t="n"/>
+      <c r="I38" s="45" t="n"/>
+      <c r="J38" s="45" t="n"/>
+      <c r="K38" s="45" t="n"/>
+      <c r="L38" s="45" t="n"/>
+      <c r="M38" s="45" t="n"/>
+      <c r="N38" s="46" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="43">
     <mergeCell ref="I34:J34"/>
-    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="N2:P2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="K31:M31"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="E9:G9"/>
     <mergeCell ref="B33:H33"/>
-    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="B37:H37"/>
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B36:H36"/>
     <mergeCell ref="K8:M8"/>
-    <mergeCell ref="B32:H32"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="J24:K24"/>
-    <mergeCell ref="I32:J32"/>
     <mergeCell ref="B35:H35"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="I37:J37"/>
     <mergeCell ref="E7:G7"/>
     <mergeCell ref="K7:M7"/>
-    <mergeCell ref="B31:H31"/>
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="H2:L2"/>
-    <mergeCell ref="N2:P3"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="H8:J8"/>
     <mergeCell ref="I33:J33"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="H28:I28"/>
     <mergeCell ref="K34:M34"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="J22:K22"/>
-    <mergeCell ref="H27:I27"/>
     <mergeCell ref="B23:H23"/>
     <mergeCell ref="K33:M33"/>
     <mergeCell ref="I35:J35"/>
     <mergeCell ref="K9:M9"/>
+    <mergeCell ref="K36:M36"/>
     <mergeCell ref="E8:G8"/>
-    <mergeCell ref="I31:J31"/>
     <mergeCell ref="K35:M35"/>
     <mergeCell ref="H9:J9"/>
     <mergeCell ref="J23:K23"/>
@@ -2007,7 +2177,7 @@
       <formula>"A_FAIRE"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K31:K35">
+  <conditionalFormatting sqref="K33:K37">
     <cfRule type="dataBar" priority="5">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -2016,7 +2186,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I31:I35">
+  <conditionalFormatting sqref="I33:I37">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
       <formula>"TERMINEE"</formula>
     </cfRule>
@@ -2132,7 +2302,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00378ADD"/>
+    <tabColor rgb="000F6E56"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2149,282 +2319,282 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="55" t="n"/>
+      <c r="B1" s="56" t="inlineStr">
         <is>
           <t>UO L09U1 — Préparation et passage des IDR</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="C1" s="55" t="n"/>
+      <c r="D1" s="55" t="n"/>
+      <c r="E1" s="55" t="n"/>
+      <c r="F1" s="55" t="n"/>
+      <c r="G1" s="55" t="n"/>
+      <c r="H1" s="55" t="n"/>
+      <c r="I1" s="55" t="n"/>
+      <c r="J1" s="55" t="n"/>
+      <c r="K1" s="57" t="inlineStr">
         <is>
           <t>Saisie — Activités · J. Dujardin</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="1" t="n"/>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>⚙  SYSTÈME : CLIMATISATION</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>▣  PROJET : PROJET DEMO</t>
+      <c r="A2" s="55" t="n"/>
+      <c r="B2" s="58" t="inlineStr">
+        <is>
+          <t>⚙  CLIMATISATION</t>
+        </is>
+      </c>
+      <c r="G2" s="55" t="n"/>
+      <c r="H2" s="58" t="inlineStr">
+        <is>
+          <t>▣  PROJET DEMO</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="1" t="n"/>
-      <c r="B3" s="6">
+      <c r="A3" s="55" t="n"/>
+      <c r="B3" s="59">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="59">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="59">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
-      <c r="H3" s="1" t="n"/>
-      <c r="I3" s="1" t="n"/>
-      <c r="J3" s="1" t="n"/>
-      <c r="K3" s="1" t="n"/>
-      <c r="L3" s="1" t="n"/>
+      <c r="H3" s="55" t="n"/>
+      <c r="I3" s="55" t="n"/>
+      <c r="J3" s="55" t="n"/>
+      <c r="K3" s="55" t="n"/>
+      <c r="L3" s="55" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1">
-      <c r="A4" s="1" t="n"/>
-      <c r="B4" s="1" t="n"/>
-      <c r="C4" s="1" t="n"/>
-      <c r="D4" s="1" t="n"/>
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="1" t="n"/>
-      <c r="H4" s="1" t="n"/>
-      <c r="I4" s="1" t="n"/>
-      <c r="J4" s="1" t="n"/>
-      <c r="K4" s="1" t="n"/>
-      <c r="L4" s="1" t="n"/>
+      <c r="A4" s="55" t="n"/>
+      <c r="B4" s="55" t="n"/>
+      <c r="C4" s="55" t="n"/>
+      <c r="D4" s="55" t="n"/>
+      <c r="E4" s="55" t="n"/>
+      <c r="F4" s="55" t="n"/>
+      <c r="G4" s="55" t="n"/>
+      <c r="H4" s="55" t="n"/>
+      <c r="I4" s="55" t="n"/>
+      <c r="J4" s="55" t="n"/>
+      <c r="K4" s="55" t="n"/>
+      <c r="L4" s="55" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="48" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B6" s="48" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>designation</t>
         </is>
       </c>
-      <c r="C6" s="48" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
-      <c r="D6" s="48" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>avancement</t>
         </is>
       </c>
-      <c r="E6" s="48" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>load (h)</t>
         </is>
       </c>
-      <c r="F6" s="48" t="inlineStr">
+      <c r="F6" s="60" t="inlineStr">
         <is>
           <t>consommé (h)</t>
         </is>
       </c>
-      <c r="G6" s="48" t="inlineStr">
+      <c r="G6" s="60" t="inlineStr">
         <is>
           <t>reste (h)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="49" t="inlineStr">
+      <c r="A7" s="61" t="inlineStr">
         <is>
           <t>ACT-01</t>
         </is>
       </c>
-      <c r="B7" s="50" t="inlineStr">
+      <c r="B7" s="62" t="inlineStr">
         <is>
           <t>Analyse fonctionnelle du besoin</t>
         </is>
       </c>
-      <c r="C7" s="49" t="inlineStr">
+      <c r="C7" s="61" t="inlineStr">
         <is>
           <t>TERMINEE</t>
         </is>
       </c>
-      <c r="D7" s="49" t="n">
+      <c r="D7" s="61" t="n">
         <v>100</v>
       </c>
-      <c r="E7" s="51" t="n">
+      <c r="E7" s="63" t="n">
         <v>24</v>
       </c>
-      <c r="F7" s="51" t="n">
+      <c r="F7" s="63" t="n">
         <v>22</v>
       </c>
-      <c r="G7" s="51" t="n">
+      <c r="G7" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="49" t="inlineStr">
+      <c r="A8" s="61" t="inlineStr">
         <is>
           <t>ACT-02</t>
         </is>
       </c>
-      <c r="B8" s="50" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>Specification des exigences</t>
         </is>
       </c>
-      <c r="C8" s="49" t="inlineStr">
+      <c r="C8" s="61" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="D8" s="49" t="n">
+      <c r="D8" s="61" t="n">
         <v>60</v>
       </c>
-      <c r="E8" s="51" t="n">
+      <c r="E8" s="63" t="n">
         <v>30</v>
       </c>
-      <c r="F8" s="51" t="n">
+      <c r="F8" s="63" t="n">
         <v>28.5</v>
       </c>
-      <c r="G8" s="51" t="n">
+      <c r="G8" s="63" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="49" t="inlineStr">
+      <c r="A9" s="61" t="inlineStr">
         <is>
           <t>ACT-03</t>
         </is>
       </c>
-      <c r="B9" s="50" t="inlineStr">
+      <c r="B9" s="62" t="inlineStr">
         <is>
           <t>Definition d'architecture</t>
         </is>
       </c>
-      <c r="C9" s="49" t="inlineStr">
+      <c r="C9" s="61" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="D9" s="49" t="n">
+      <c r="D9" s="61" t="n">
         <v>35</v>
       </c>
-      <c r="E9" s="51" t="n">
+      <c r="E9" s="63" t="n">
         <v>40</v>
       </c>
-      <c r="F9" s="51" t="n">
+      <c r="F9" s="63" t="n">
         <v>12</v>
       </c>
-      <c r="G9" s="51" t="n">
+      <c r="G9" s="63" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="49" t="inlineStr">
+      <c r="A10" s="61" t="inlineStr">
         <is>
           <t>ACT-04</t>
         </is>
       </c>
-      <c r="B10" s="50" t="inlineStr">
+      <c r="B10" s="62" t="inlineStr">
         <is>
           <t>Calculs et simulations</t>
         </is>
       </c>
-      <c r="C10" s="49" t="inlineStr">
+      <c r="C10" s="61" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="D10" s="49" t="n">
+      <c r="D10" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="51" t="n">
+      <c r="E10" s="63" t="n">
         <v>35</v>
       </c>
-      <c r="F10" s="51" t="n">
+      <c r="F10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="51" t="n">
+      <c r="G10" s="63" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="49" t="inlineStr">
+      <c r="A11" s="61" t="inlineStr">
         <is>
           <t>ACT-05</t>
         </is>
       </c>
-      <c r="B11" s="50" t="inlineStr">
+      <c r="B11" s="62" t="inlineStr">
         <is>
           <t>Revue de conception</t>
         </is>
       </c>
-      <c r="C11" s="49" t="inlineStr">
+      <c r="C11" s="61" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="D11" s="49" t="n">
+      <c r="D11" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="51" t="n">
+      <c r="E11" s="63" t="n">
         <v>25</v>
       </c>
-      <c r="F11" s="51" t="n">
+      <c r="F11" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="51" t="n">
+      <c r="G11" s="63" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="49" t="inlineStr">
+      <c r="A12" s="61" t="inlineStr">
         <is>
           <t>ACT-06</t>
         </is>
       </c>
-      <c r="B12" s="50" t="inlineStr">
+      <c r="B12" s="62" t="inlineStr">
         <is>
           <t>Preparation gate review</t>
         </is>
       </c>
-      <c r="C12" s="49" t="inlineStr">
+      <c r="C12" s="61" t="inlineStr">
         <is>
           <t>STAND_BY</t>
         </is>
       </c>
-      <c r="D12" s="49" t="n">
+      <c r="D12" s="61" t="n">
         <v>10</v>
       </c>
-      <c r="E12" s="51" t="n">
+      <c r="E12" s="63" t="n">
         <v>46</v>
       </c>
-      <c r="F12" s="51" t="n">
+      <c r="F12" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="51" t="n">
+      <c r="G12" s="63" t="n">
         <v>41.4</v>
       </c>
     </row>
@@ -2467,7 +2637,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00EF9F27"/>
+    <tabColor rgb="00BA7517"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2482,173 +2652,173 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="A1" s="64" t="n"/>
+      <c r="B1" s="65" t="inlineStr">
         <is>
           <t>UO L09U1 — Préparation et passage des IDR</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="52" t="inlineStr">
+      <c r="C1" s="64" t="n"/>
+      <c r="D1" s="64" t="n"/>
+      <c r="E1" s="64" t="n"/>
+      <c r="F1" s="64" t="n"/>
+      <c r="G1" s="64" t="n"/>
+      <c r="H1" s="64" t="n"/>
+      <c r="I1" s="64" t="n"/>
+      <c r="J1" s="64" t="n"/>
+      <c r="K1" s="66" t="inlineStr">
         <is>
           <t>Points ouverts — OIL · J. Dujardin</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="1" t="n"/>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>⚙  SYSTÈME : CLIMATISATION</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>▣  PROJET : PROJET DEMO</t>
+      <c r="A2" s="64" t="n"/>
+      <c r="B2" s="67" t="inlineStr">
+        <is>
+          <t>⚙  CLIMATISATION</t>
+        </is>
+      </c>
+      <c r="G2" s="64" t="n"/>
+      <c r="H2" s="67" t="inlineStr">
+        <is>
+          <t>▣  PROJET DEMO</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="1" t="n"/>
-      <c r="B3" s="6">
+      <c r="A3" s="64" t="n"/>
+      <c r="B3" s="68">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="68">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="68">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
-      <c r="H3" s="1" t="n"/>
-      <c r="I3" s="1" t="n"/>
-      <c r="J3" s="1" t="n"/>
+      <c r="H3" s="64" t="n"/>
+      <c r="I3" s="64" t="n"/>
+      <c r="J3" s="64" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1">
-      <c r="A4" s="1" t="n"/>
-      <c r="B4" s="1" t="n"/>
-      <c r="C4" s="1" t="n"/>
-      <c r="D4" s="1" t="n"/>
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="1" t="n"/>
-      <c r="H4" s="1" t="n"/>
-      <c r="I4" s="1" t="n"/>
-      <c r="J4" s="1" t="n"/>
+      <c r="A4" s="64" t="n"/>
+      <c r="B4" s="64" t="n"/>
+      <c r="C4" s="64" t="n"/>
+      <c r="D4" s="64" t="n"/>
+      <c r="E4" s="64" t="n"/>
+      <c r="F4" s="64" t="n"/>
+      <c r="G4" s="64" t="n"/>
+      <c r="H4" s="64" t="n"/>
+      <c r="I4" s="64" t="n"/>
+      <c r="J4" s="64" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="48" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B6" s="48" t="inlineStr">
+      <c r="B6" s="60" t="inlineStr">
         <is>
           <t>titre</t>
         </is>
       </c>
-      <c r="C6" s="48" t="inlineStr">
+      <c r="C6" s="60" t="inlineStr">
         <is>
           <t>en_action</t>
         </is>
       </c>
-      <c r="D6" s="48" t="inlineStr">
+      <c r="D6" s="60" t="inlineStr">
         <is>
           <t>criticite</t>
         </is>
       </c>
-      <c r="E6" s="48" t="inlineStr">
+      <c r="E6" s="60" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="49" t="inlineStr">
+      <c r="A7" s="61" t="inlineStr">
         <is>
           <t>PO-001</t>
         </is>
       </c>
-      <c r="B7" s="50" t="inlineStr">
+      <c r="B7" s="62" t="inlineStr">
         <is>
           <t>Question expert normes EN 45545</t>
         </is>
       </c>
-      <c r="C7" s="49" t="inlineStr">
+      <c r="C7" s="61" t="inlineStr">
         <is>
           <t>EXPERT</t>
         </is>
       </c>
-      <c r="D7" s="49" t="inlineStr">
+      <c r="D7" s="61" t="inlineStr">
         <is>
           <t>HAUTE</t>
         </is>
       </c>
-      <c r="E7" s="49" t="inlineStr">
+      <c r="E7" s="61" t="inlineStr">
         <is>
           <t>OUVERT</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="49" t="inlineStr">
+      <c r="A8" s="61" t="inlineStr">
         <is>
           <t>PO-002</t>
         </is>
       </c>
-      <c r="B8" s="50" t="inlineStr">
+      <c r="B8" s="62" t="inlineStr">
         <is>
           <t>Attente retour relecture fournisseur</t>
         </is>
       </c>
-      <c r="C8" s="49" t="inlineStr">
+      <c r="C8" s="61" t="inlineStr">
         <is>
           <t>FOURNISSEUR</t>
         </is>
       </c>
-      <c r="D8" s="49" t="inlineStr">
+      <c r="D8" s="61" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
-      <c r="E8" s="49" t="inlineStr">
+      <c r="E8" s="61" t="inlineStr">
         <is>
           <t>OUVERT</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="49" t="inlineStr">
+      <c r="A9" s="61" t="inlineStr">
         <is>
           <t>PO-003</t>
         </is>
       </c>
-      <c r="B9" s="50" t="inlineStr">
+      <c r="B9" s="62" t="inlineStr">
         <is>
           <t>Acces outil documentaire obtenu</t>
         </is>
       </c>
-      <c r="C9" s="49" t="inlineStr">
+      <c r="C9" s="61" t="inlineStr">
         <is>
           <t>SE</t>
         </is>
       </c>
-      <c r="D9" s="49" t="inlineStr">
+      <c r="D9" s="61" t="inlineStr">
         <is>
           <t>BASSE</t>
         </is>
       </c>
-      <c r="E9" s="49" t="inlineStr">
+      <c r="E9" s="61" t="inlineStr">
         <is>
           <t>CLOS</t>
         </is>

</xml_diff>

<commit_message>
feat(design): Design B v4 — rendu verifie visuellement via Excel COM
- Camemberts : plus de titre superpose, libelles en cellules sous chaque
  anneau (Avancement - 45 %...)
- Alignement : tout le Dashboard (cartes, camemberts, 3 zones) cale sur
  la largeur exacte du bandeau (colonnes B..P)
- Chips supprimees : CLIMATISATION - PROJET DEMO en texte simple sous le
  titre, meme fond que le bandeau
- Bandeau = largeur exacte du contenu sur chaque feuille (ne deborde
  plus) ; navigation adaptative sur feuilles etroites
- Harmonie par onglet : en-tetes de tableaux de la couleur du bandeau
  (Dashboard marine, Activites teal, OIL ambre)
- Rendu controle par export PDF Excel reel (3 pages inspectees)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projet_TrainSystem/Design_B_Cockpit.xlsx
+++ b/projet_TrainSystem/Design_B_Cockpit.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,11 +38,6 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00B5D4F4"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
@@ -50,6 +45,11 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="00B5D4F4"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="00B5D4F4"/>
       <sz val="9"/>
     </font>
@@ -98,17 +98,17 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000C447C"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="002C2C2A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="000C447C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002C2C2A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -142,11 +142,6 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="009FE1CB"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="009FE1CB"/>
       <sz val="9"/>
@@ -159,17 +154,12 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00FAC775"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FAC775"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -179,11 +169,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000C447C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00185FA5"/>
       </patternFill>
     </fill>
     <fill>
@@ -223,21 +208,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00085041"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00BA7517"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00854F0B"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="43">
+  <borders count="44">
     <border>
       <left/>
       <right/>
@@ -624,6 +599,15 @@
       <bottom style="thin">
         <color rgb="00D3D1C7"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D1C7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -643,134 +627,150 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -928,21 +928,6 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Avancement — 45 %</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
     <plotArea>
       <doughnutChart>
         <varyColors val="1"/>
@@ -995,21 +980,6 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Heures — 30 %</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
     <plotArea>
       <doughnutChart>
         <varyColors val="1"/>
@@ -1062,21 +1032,6 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Livrables — 33 %</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
     <plotArea>
       <doughnutChart>
         <varyColors val="1"/>
@@ -1129,21 +1084,6 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Données d'entrée — 67 %</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
     <plotArea>
       <doughnutChart>
         <varyColors val="1"/>
@@ -1219,7 +1159,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>10</row>
       <rowOff>0</rowOff>
@@ -1241,7 +1181,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>9</col>
       <colOff>0</colOff>
       <row>10</row>
       <rowOff>0</rowOff>
@@ -1263,7 +1203,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>10</row>
       <rowOff>0</rowOff>
@@ -1576,7 +1516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q38"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1605,57 +1545,32 @@
           <t>UO L09U1 — Préparation et passage des IDR</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>Cockpit de pilotage · J. Dujardin</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
       <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="1" t="n"/>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>⚙  CLIMATISATION</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>▣  PROJET DEMO</t>
-        </is>
-      </c>
-      <c r="M2" s="1" t="n"/>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>CLIMATISATION  —  PROJET DEMO</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>SANTÉ ROUGE</t>
         </is>
       </c>
-      <c r="Q2" s="1" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="6">
+      <c r="B3" s="5">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
@@ -1665,10 +1580,11 @@
       <c r="K3" s="1" t="n"/>
       <c r="L3" s="1" t="n"/>
       <c r="M3" s="1" t="n"/>
-      <c r="N3" s="1" t="n"/>
-      <c r="O3" s="1" t="n"/>
-      <c r="P3" s="1" t="n"/>
-      <c r="Q3" s="1" t="n"/>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Cockpit de pilotage · J. Dujardin</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="6" customHeight="1">
       <c r="A4" s="1" t="n"/>
@@ -1687,21 +1603,20 @@
       <c r="N4" s="1" t="n"/>
       <c r="O4" s="1" t="n"/>
       <c r="P4" s="1" t="n"/>
-      <c r="Q4" s="1" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="B6" s="7" t="n"/>
       <c r="C6" s="8" t="n"/>
       <c r="D6" s="9" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="13" t="n"/>
-      <c r="I6" s="14" t="n"/>
-      <c r="J6" s="15" t="n"/>
-      <c r="K6" s="10" t="n"/>
-      <c r="L6" s="11" t="n"/>
-      <c r="M6" s="12" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="12" t="n"/>
+      <c r="J6" s="13" t="n"/>
+      <c r="K6" s="14" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="N6" s="10" t="n"/>
+      <c r="O6" s="11" t="n"/>
+      <c r="P6" s="12" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="16" t="inlineStr">
@@ -1710,24 +1625,24 @@
         </is>
       </c>
       <c r="D7" s="17" t="n"/>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>CONSOMMÉ</t>
         </is>
       </c>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="H7" s="19" t="n"/>
+      <c r="J7" s="20" t="inlineStr">
         <is>
           <t>POINTS OUVERTS</t>
         </is>
       </c>
-      <c r="J7" s="21" t="n"/>
-      <c r="K7" s="18" t="inlineStr">
+      <c r="L7" s="21" t="n"/>
+      <c r="N7" s="18" t="inlineStr">
         <is>
           <t>EAC</t>
         </is>
       </c>
-      <c r="M7" s="19" t="n"/>
+      <c r="P7" s="19" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="22" t="inlineStr">
@@ -1736,24 +1651,24 @@
         </is>
       </c>
       <c r="D8" s="17" t="n"/>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="F8" s="23" t="inlineStr">
         <is>
           <t>29,5 %</t>
         </is>
       </c>
-      <c r="G8" s="19" t="n"/>
-      <c r="H8" s="24" t="inlineStr">
+      <c r="H8" s="19" t="n"/>
+      <c r="J8" s="24" t="inlineStr">
         <is>
           <t>2  ▲1</t>
         </is>
       </c>
-      <c r="J8" s="21" t="n"/>
-      <c r="K8" s="25" t="inlineStr">
+      <c r="L8" s="21" t="n"/>
+      <c r="N8" s="25" t="inlineStr">
         <is>
           <t>169 h</t>
         </is>
       </c>
-      <c r="M8" s="19" t="n"/>
+      <c r="P8" s="19" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="26" t="inlineStr">
@@ -1763,407 +1678,448 @@
       </c>
       <c r="C9" s="27" t="n"/>
       <c r="D9" s="28" t="n"/>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="F9" s="29" t="inlineStr">
         <is>
           <t>59 h / 200 h</t>
         </is>
       </c>
-      <c r="F9" s="30" t="n"/>
-      <c r="G9" s="31" t="n"/>
-      <c r="H9" s="32" t="inlineStr">
+      <c r="G9" s="30" t="n"/>
+      <c r="H9" s="31" t="n"/>
+      <c r="J9" s="32" t="inlineStr">
         <is>
           <t>dont 1 critique</t>
         </is>
       </c>
-      <c r="I9" s="33" t="n"/>
-      <c r="J9" s="34" t="n"/>
-      <c r="K9" s="29" t="inlineStr">
+      <c r="K9" s="33" t="n"/>
+      <c r="L9" s="34" t="n"/>
+      <c r="N9" s="29" t="inlineStr">
         <is>
           <t>dérive −31 h</t>
         </is>
       </c>
-      <c r="L9" s="30" t="n"/>
-      <c r="M9" s="31" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="35" t="inlineStr">
+      <c r="O9" s="30" t="n"/>
+      <c r="P9" s="31" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>Avancement — 45 %</t>
+        </is>
+      </c>
+      <c r="F20" s="35" t="inlineStr">
+        <is>
+          <t>Heures — 30 %</t>
+        </is>
+      </c>
+      <c r="J20" s="35" t="inlineStr">
+        <is>
+          <t>Livrables — 33 %</t>
+        </is>
+      </c>
+      <c r="N20" s="35" t="inlineStr">
+        <is>
+          <t>Données d'entrée — 67 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t>Prochains livrables</t>
         </is>
       </c>
-      <c r="C21" s="36" t="n"/>
-      <c r="D21" s="36" t="n"/>
-      <c r="E21" s="36" t="n"/>
-      <c r="F21" s="36" t="n"/>
-      <c r="G21" s="36" t="n"/>
-      <c r="H21" s="36" t="n"/>
-      <c r="I21" s="36" t="n"/>
-      <c r="J21" s="36" t="n"/>
-      <c r="K21" s="36" t="n"/>
-      <c r="L21" s="36" t="n"/>
-      <c r="M21" s="36" t="n"/>
-      <c r="N21" s="37" t="n"/>
-    </row>
-    <row r="22" ht="19" customHeight="1">
-      <c r="B22" s="38" t="inlineStr">
+      <c r="C22" s="37" t="n"/>
+      <c r="D22" s="37" t="n"/>
+      <c r="E22" s="37" t="n"/>
+      <c r="F22" s="37" t="n"/>
+      <c r="G22" s="37" t="n"/>
+      <c r="H22" s="37" t="n"/>
+      <c r="I22" s="37" t="n"/>
+      <c r="J22" s="37" t="n"/>
+      <c r="K22" s="37" t="n"/>
+      <c r="L22" s="37" t="n"/>
+      <c r="M22" s="37" t="n"/>
+      <c r="N22" s="37" t="n"/>
+      <c r="O22" s="37" t="n"/>
+      <c r="P22" s="38" t="n"/>
+    </row>
+    <row r="23" ht="19" customHeight="1">
+      <c r="B23" s="39" t="inlineStr">
         <is>
           <t>SAA.RS — Requirement Spec</t>
         </is>
       </c>
-      <c r="C22" s="39" t="n"/>
-      <c r="D22" s="39" t="n"/>
-      <c r="E22" s="39" t="n"/>
-      <c r="F22" s="39" t="n"/>
-      <c r="G22" s="39" t="n"/>
-      <c r="H22" s="39" t="n"/>
-      <c r="I22" s="40" t="inlineStr">
+      <c r="C23" s="40" t="n"/>
+      <c r="D23" s="40" t="n"/>
+      <c r="E23" s="40" t="n"/>
+      <c r="F23" s="40" t="n"/>
+      <c r="G23" s="40" t="n"/>
+      <c r="H23" s="40" t="n"/>
+      <c r="I23" s="40" t="n"/>
+      <c r="J23" s="40" t="n"/>
+      <c r="K23" s="40" t="n"/>
+      <c r="L23" s="41" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="J22" s="41" t="inlineStr">
+      <c r="M23" s="42" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="K22" s="39" t="n"/>
-      <c r="L22" s="42" t="n"/>
-      <c r="M22" s="42" t="n"/>
-      <c r="N22" s="43" t="n"/>
-    </row>
-    <row r="23" ht="19" customHeight="1">
-      <c r="B23" s="38" t="inlineStr">
+      <c r="N23" s="40" t="n"/>
+      <c r="O23" s="40" t="n"/>
+      <c r="P23" s="43" t="n"/>
+    </row>
+    <row r="24" ht="19" customHeight="1">
+      <c r="B24" s="39" t="inlineStr">
         <is>
           <t>RSS.RS — Subsystem Spec</t>
         </is>
       </c>
-      <c r="C23" s="39" t="n"/>
-      <c r="D23" s="39" t="n"/>
-      <c r="E23" s="39" t="n"/>
-      <c r="F23" s="39" t="n"/>
-      <c r="G23" s="39" t="n"/>
-      <c r="H23" s="39" t="n"/>
-      <c r="I23" s="40" t="inlineStr">
+      <c r="C24" s="40" t="n"/>
+      <c r="D24" s="40" t="n"/>
+      <c r="E24" s="40" t="n"/>
+      <c r="F24" s="40" t="n"/>
+      <c r="G24" s="40" t="n"/>
+      <c r="H24" s="40" t="n"/>
+      <c r="I24" s="40" t="n"/>
+      <c r="J24" s="40" t="n"/>
+      <c r="K24" s="40" t="n"/>
+      <c r="L24" s="41" t="inlineStr">
         <is>
           <t>M3</t>
         </is>
       </c>
-      <c r="J23" s="41" t="inlineStr">
+      <c r="M24" s="42" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K23" s="39" t="n"/>
-      <c r="L23" s="42" t="n"/>
-      <c r="M23" s="42" t="n"/>
-      <c r="N23" s="43" t="n"/>
-    </row>
-    <row r="24" ht="19" customHeight="1">
-      <c r="B24" s="38" t="inlineStr">
+      <c r="N24" s="40" t="n"/>
+      <c r="O24" s="40" t="n"/>
+      <c r="P24" s="43" t="n"/>
+    </row>
+    <row r="25" ht="19" customHeight="1">
+      <c r="B25" s="39" t="inlineStr">
         <is>
           <t>DR.RS — Design Review file</t>
         </is>
       </c>
-      <c r="C24" s="39" t="n"/>
-      <c r="D24" s="39" t="n"/>
-      <c r="E24" s="39" t="n"/>
-      <c r="F24" s="39" t="n"/>
-      <c r="G24" s="39" t="n"/>
-      <c r="H24" s="39" t="n"/>
-      <c r="I24" s="40" t="inlineStr">
+      <c r="C25" s="40" t="n"/>
+      <c r="D25" s="40" t="n"/>
+      <c r="E25" s="40" t="n"/>
+      <c r="F25" s="40" t="n"/>
+      <c r="G25" s="40" t="n"/>
+      <c r="H25" s="40" t="n"/>
+      <c r="I25" s="40" t="n"/>
+      <c r="J25" s="40" t="n"/>
+      <c r="K25" s="40" t="n"/>
+      <c r="L25" s="41" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J24" s="41" t="inlineStr">
+      <c r="M25" s="42" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K24" s="39" t="n"/>
-      <c r="L24" s="42" t="n"/>
-      <c r="M24" s="42" t="n"/>
-      <c r="N24" s="43" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="44" t="n"/>
-      <c r="C25" s="45" t="n"/>
-      <c r="D25" s="45" t="n"/>
-      <c r="E25" s="45" t="n"/>
-      <c r="F25" s="45" t="n"/>
-      <c r="G25" s="45" t="n"/>
-      <c r="H25" s="45" t="n"/>
-      <c r="I25" s="45" t="n"/>
-      <c r="J25" s="45" t="n"/>
-      <c r="K25" s="45" t="n"/>
-      <c r="L25" s="45" t="n"/>
-      <c r="M25" s="45" t="n"/>
-      <c r="N25" s="46" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="35" t="inlineStr">
+      <c r="N25" s="40" t="n"/>
+      <c r="O25" s="40" t="n"/>
+      <c r="P25" s="43" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="44" t="n"/>
+      <c r="C26" s="45" t="n"/>
+      <c r="D26" s="45" t="n"/>
+      <c r="E26" s="45" t="n"/>
+      <c r="F26" s="45" t="n"/>
+      <c r="G26" s="45" t="n"/>
+      <c r="H26" s="45" t="n"/>
+      <c r="I26" s="45" t="n"/>
+      <c r="J26" s="45" t="n"/>
+      <c r="K26" s="45" t="n"/>
+      <c r="L26" s="45" t="n"/>
+      <c r="M26" s="45" t="n"/>
+      <c r="N26" s="45" t="n"/>
+      <c r="O26" s="45" t="n"/>
+      <c r="P26" s="46" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="36" t="inlineStr">
         <is>
           <t>La balle est chez…</t>
         </is>
       </c>
-      <c r="C27" s="36" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
-      <c r="F27" s="36" t="n"/>
-      <c r="G27" s="36" t="n"/>
-      <c r="H27" s="36" t="n"/>
-      <c r="I27" s="36" t="n"/>
-      <c r="J27" s="36" t="n"/>
-      <c r="K27" s="36" t="n"/>
-      <c r="L27" s="36" t="n"/>
-      <c r="M27" s="36" t="n"/>
-      <c r="N27" s="37" t="n"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="47" t="inlineStr">
+      <c r="C28" s="37" t="n"/>
+      <c r="D28" s="37" t="n"/>
+      <c r="E28" s="37" t="n"/>
+      <c r="F28" s="37" t="n"/>
+      <c r="G28" s="37" t="n"/>
+      <c r="H28" s="37" t="n"/>
+      <c r="I28" s="37" t="n"/>
+      <c r="J28" s="37" t="n"/>
+      <c r="K28" s="37" t="n"/>
+      <c r="L28" s="37" t="n"/>
+      <c r="M28" s="37" t="n"/>
+      <c r="N28" s="37" t="n"/>
+      <c r="O28" s="37" t="n"/>
+      <c r="P28" s="38" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="47" t="inlineStr">
         <is>
           <t>FOURNISSEUR : 1</t>
         </is>
       </c>
-      <c r="D28" s="42" t="n"/>
-      <c r="E28" s="48" t="inlineStr">
+      <c r="F29" s="48" t="n"/>
+      <c r="G29" s="49" t="inlineStr">
         <is>
           <t>EXPERT : 1</t>
         </is>
       </c>
-      <c r="G28" s="42" t="n"/>
-      <c r="H28" s="49" t="inlineStr">
+      <c r="K29" s="48" t="n"/>
+      <c r="L29" s="50" t="inlineStr">
         <is>
           <t>NOUS (SE) : 0</t>
         </is>
       </c>
-      <c r="J28" s="42" t="n"/>
-      <c r="K28" s="42" t="n"/>
-      <c r="L28" s="42" t="n"/>
-      <c r="M28" s="42" t="n"/>
-      <c r="N28" s="43" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="44" t="n"/>
-      <c r="C29" s="45" t="n"/>
-      <c r="D29" s="45" t="n"/>
-      <c r="E29" s="45" t="n"/>
-      <c r="F29" s="45" t="n"/>
-      <c r="G29" s="45" t="n"/>
-      <c r="H29" s="45" t="n"/>
-      <c r="I29" s="45" t="n"/>
-      <c r="J29" s="45" t="n"/>
-      <c r="K29" s="45" t="n"/>
-      <c r="L29" s="45" t="n"/>
-      <c r="M29" s="45" t="n"/>
-      <c r="N29" s="46" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="35" t="inlineStr">
+      <c r="P29" s="43" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="44" t="n"/>
+      <c r="C30" s="45" t="n"/>
+      <c r="D30" s="45" t="n"/>
+      <c r="E30" s="45" t="n"/>
+      <c r="F30" s="45" t="n"/>
+      <c r="G30" s="45" t="n"/>
+      <c r="H30" s="45" t="n"/>
+      <c r="I30" s="45" t="n"/>
+      <c r="J30" s="45" t="n"/>
+      <c r="K30" s="45" t="n"/>
+      <c r="L30" s="45" t="n"/>
+      <c r="M30" s="45" t="n"/>
+      <c r="N30" s="45" t="n"/>
+      <c r="O30" s="45" t="n"/>
+      <c r="P30" s="46" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="36" t="inlineStr">
         <is>
           <t>Avancement des activités en cours</t>
         </is>
       </c>
-      <c r="C31" s="36" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="36" t="n"/>
-      <c r="G31" s="36" t="n"/>
-      <c r="H31" s="36" t="n"/>
-      <c r="I31" s="50" t="inlineStr">
+      <c r="C32" s="37" t="n"/>
+      <c r="D32" s="37" t="n"/>
+      <c r="E32" s="37" t="n"/>
+      <c r="F32" s="37" t="n"/>
+      <c r="G32" s="37" t="n"/>
+      <c r="H32" s="37" t="n"/>
+      <c r="I32" s="37" t="n"/>
+      <c r="J32" s="51" t="inlineStr">
         <is>
           <t>(les activités terminées ne sont pas affichées)</t>
         </is>
       </c>
-      <c r="J31" s="36" t="n"/>
-      <c r="K31" s="36" t="n"/>
-      <c r="L31" s="36" t="n"/>
-      <c r="M31" s="36" t="n"/>
-      <c r="N31" s="37" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="51" t="inlineStr">
+      <c r="K32" s="52" t="n"/>
+      <c r="L32" s="52" t="n"/>
+      <c r="M32" s="52" t="n"/>
+      <c r="N32" s="52" t="n"/>
+      <c r="O32" s="52" t="n"/>
+      <c r="P32" s="38" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="53" t="inlineStr">
         <is>
           <t>activité</t>
         </is>
       </c>
-      <c r="C32" s="39" t="n"/>
-      <c r="D32" s="39" t="n"/>
-      <c r="E32" s="39" t="n"/>
-      <c r="F32" s="39" t="n"/>
-      <c r="G32" s="39" t="n"/>
-      <c r="H32" s="39" t="n"/>
-      <c r="I32" s="51" t="inlineStr">
+      <c r="C33" s="40" t="n"/>
+      <c r="D33" s="40" t="n"/>
+      <c r="E33" s="40" t="n"/>
+      <c r="F33" s="40" t="n"/>
+      <c r="G33" s="40" t="n"/>
+      <c r="H33" s="40" t="n"/>
+      <c r="I33" s="40" t="n"/>
+      <c r="J33" s="53" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
-      <c r="J32" s="39" t="n"/>
-      <c r="K32" s="51" t="inlineStr">
+      <c r="K33" s="40" t="n"/>
+      <c r="L33" s="53" t="inlineStr">
         <is>
           <t>avancement</t>
         </is>
       </c>
-      <c r="L32" s="39" t="n"/>
-      <c r="M32" s="39" t="n"/>
-      <c r="N32" s="51" t="inlineStr">
+      <c r="M33" s="40" t="n"/>
+      <c r="N33" s="40" t="n"/>
+      <c r="O33" s="53" t="inlineStr">
         <is>
           <t>heures</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="B33" s="52" t="inlineStr">
+      <c r="P33" s="40" t="n"/>
+    </row>
+    <row r="34" ht="19" customHeight="1">
+      <c r="B34" s="54" t="inlineStr">
         <is>
           <t>ACT-02 — Specification des exigences</t>
         </is>
       </c>
-      <c r="I33" s="53" t="inlineStr">
+      <c r="J34" s="55" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="K33" s="53" t="n">
+      <c r="L34" s="55" t="n">
         <v>60</v>
       </c>
-      <c r="N33" s="54" t="n">
+      <c r="O34" s="56" t="n">
         <v>28.5</v>
       </c>
-    </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="B34" s="52" t="inlineStr">
+      <c r="P34" s="43" t="n"/>
+    </row>
+    <row r="35" ht="19" customHeight="1">
+      <c r="B35" s="54" t="inlineStr">
         <is>
           <t>ACT-03 — Definition d'architecture</t>
         </is>
       </c>
-      <c r="I34" s="53" t="inlineStr">
+      <c r="J35" s="55" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="K34" s="53" t="n">
+      <c r="L35" s="55" t="n">
         <v>35</v>
       </c>
-      <c r="N34" s="54" t="n">
+      <c r="O35" s="56" t="n">
         <v>12</v>
       </c>
-    </row>
-    <row r="35" ht="19" customHeight="1">
-      <c r="B35" s="52" t="inlineStr">
+      <c r="P35" s="43" t="n"/>
+    </row>
+    <row r="36" ht="19" customHeight="1">
+      <c r="B36" s="54" t="inlineStr">
         <is>
           <t>ACT-04 — Calculs et simulations</t>
         </is>
       </c>
-      <c r="I35" s="53" t="inlineStr">
+      <c r="J36" s="55" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K35" s="53" t="n">
+      <c r="L36" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="N35" s="54" t="n">
+      <c r="O36" s="56" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" ht="19" customHeight="1">
-      <c r="B36" s="52" t="inlineStr">
+      <c r="P36" s="43" t="n"/>
+    </row>
+    <row r="37" ht="19" customHeight="1">
+      <c r="B37" s="54" t="inlineStr">
         <is>
           <t>ACT-05 — Revue de conception</t>
         </is>
       </c>
-      <c r="I36" s="53" t="inlineStr">
+      <c r="J37" s="55" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="K36" s="53" t="n">
+      <c r="L37" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="N36" s="54" t="n">
+      <c r="O37" s="56" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" ht="19" customHeight="1">
-      <c r="B37" s="52" t="inlineStr">
+      <c r="P37" s="43" t="n"/>
+    </row>
+    <row r="38" ht="19" customHeight="1">
+      <c r="B38" s="57" t="inlineStr">
         <is>
           <t>ACT-06 — Preparation gate review</t>
         </is>
       </c>
-      <c r="I37" s="53" t="inlineStr">
+      <c r="C38" s="30" t="n"/>
+      <c r="D38" s="30" t="n"/>
+      <c r="E38" s="30" t="n"/>
+      <c r="F38" s="30" t="n"/>
+      <c r="G38" s="30" t="n"/>
+      <c r="H38" s="30" t="n"/>
+      <c r="I38" s="30" t="n"/>
+      <c r="J38" s="58" t="inlineStr">
         <is>
           <t>STAND_BY</t>
         </is>
       </c>
-      <c r="K37" s="53" t="n">
+      <c r="K38" s="30" t="n"/>
+      <c r="L38" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="N37" s="54" t="n">
+      <c r="M38" s="30" t="n"/>
+      <c r="N38" s="30" t="n"/>
+      <c r="O38" s="59" t="n">
         <v>4</v>
       </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="44" t="n"/>
-      <c r="C38" s="45" t="n"/>
-      <c r="D38" s="45" t="n"/>
-      <c r="E38" s="45" t="n"/>
-      <c r="F38" s="45" t="n"/>
-      <c r="G38" s="45" t="n"/>
-      <c r="H38" s="45" t="n"/>
-      <c r="I38" s="45" t="n"/>
-      <c r="J38" s="45" t="n"/>
-      <c r="K38" s="45" t="n"/>
-      <c r="L38" s="45" t="n"/>
-      <c r="M38" s="45" t="n"/>
-      <c r="N38" s="46" t="n"/>
+      <c r="P38" s="46" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="43">
-    <mergeCell ref="I34:J34"/>
+  <mergeCells count="48">
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="B2:M2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="B3:C3"/>
+    <mergeCell ref="L29:O29"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="B37:H37"/>
-    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="L35:N35"/>
     <mergeCell ref="F3:G3"/>
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="K8:M8"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="B35:H35"/>
-    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="L38:N38"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="J32:O32"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="K7:M7"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="K37:M37"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="B25:K25"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B1:O1"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="B37:I37"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="K33:M33"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="K9:M9"/>
-    <mergeCell ref="K36:M36"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="K35:M35"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="B23:K23"/>
+    <mergeCell ref="L37:N37"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="N3:P3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J22:J24">
+  <conditionalFormatting sqref="M23:M25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"TERMINEE"</formula>
     </cfRule>
@@ -2177,7 +2133,7 @@
       <formula>"A_FAIRE"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K33:K37">
+  <conditionalFormatting sqref="L34:L38">
     <cfRule type="dataBar" priority="5">
       <dataBar showValue="1">
         <cfvo type="num" val="0"/>
@@ -2186,7 +2142,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I33:I37">
+  <conditionalFormatting sqref="J34:J38">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
       <formula>"TERMINEE"</formula>
     </cfRule>
@@ -2306,7 +2262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2319,293 +2275,265 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="55" t="n"/>
-      <c r="B1" s="56" t="inlineStr">
+      <c r="A1" s="60" t="n"/>
+      <c r="B1" s="61" t="inlineStr">
         <is>
           <t>UO L09U1 — Préparation et passage des IDR</t>
         </is>
       </c>
-      <c r="C1" s="55" t="n"/>
-      <c r="D1" s="55" t="n"/>
-      <c r="E1" s="55" t="n"/>
-      <c r="F1" s="55" t="n"/>
-      <c r="G1" s="55" t="n"/>
-      <c r="H1" s="55" t="n"/>
-      <c r="I1" s="55" t="n"/>
-      <c r="J1" s="55" t="n"/>
-      <c r="K1" s="57" t="inlineStr">
-        <is>
-          <t>Saisie — Activités · J. Dujardin</t>
-        </is>
-      </c>
+      <c r="G1" s="60" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="55" t="n"/>
-      <c r="B2" s="58" t="inlineStr">
-        <is>
-          <t>⚙  CLIMATISATION</t>
-        </is>
-      </c>
-      <c r="G2" s="55" t="n"/>
-      <c r="H2" s="58" t="inlineStr">
-        <is>
-          <t>▣  PROJET DEMO</t>
-        </is>
-      </c>
+      <c r="A2" s="60" t="n"/>
+      <c r="B2" s="62" t="inlineStr">
+        <is>
+          <t>CLIMATISATION  —  PROJET DEMO</t>
+        </is>
+      </c>
+      <c r="G2" s="60" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="55" t="n"/>
-      <c r="B3" s="59">
+      <c r="A3" s="60" t="n"/>
+      <c r="B3" s="63">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="59">
+      <c r="C3" s="63">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="59">
+      <c r="D3" s="63">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
-      <c r="H3" s="55" t="n"/>
-      <c r="I3" s="55" t="n"/>
-      <c r="J3" s="55" t="n"/>
-      <c r="K3" s="55" t="n"/>
-      <c r="L3" s="55" t="n"/>
+      <c r="E3" s="60" t="n"/>
+      <c r="F3" s="60" t="n"/>
+      <c r="G3" s="60" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1">
-      <c r="A4" s="55" t="n"/>
-      <c r="B4" s="55" t="n"/>
-      <c r="C4" s="55" t="n"/>
-      <c r="D4" s="55" t="n"/>
-      <c r="E4" s="55" t="n"/>
-      <c r="F4" s="55" t="n"/>
-      <c r="G4" s="55" t="n"/>
-      <c r="H4" s="55" t="n"/>
-      <c r="I4" s="55" t="n"/>
-      <c r="J4" s="55" t="n"/>
-      <c r="K4" s="55" t="n"/>
-      <c r="L4" s="55" t="n"/>
+      <c r="A4" s="60" t="n"/>
+      <c r="B4" s="60" t="n"/>
+      <c r="C4" s="60" t="n"/>
+      <c r="D4" s="60" t="n"/>
+      <c r="E4" s="60" t="n"/>
+      <c r="F4" s="60" t="n"/>
+      <c r="G4" s="60" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="64" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="64" t="inlineStr">
         <is>
           <t>designation</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="64" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="64" t="inlineStr">
         <is>
           <t>avancement</t>
         </is>
       </c>
-      <c r="E6" s="60" t="inlineStr">
+      <c r="E6" s="64" t="inlineStr">
         <is>
           <t>load (h)</t>
         </is>
       </c>
-      <c r="F6" s="60" t="inlineStr">
+      <c r="F6" s="64" t="inlineStr">
         <is>
           <t>consommé (h)</t>
         </is>
       </c>
-      <c r="G6" s="60" t="inlineStr">
+      <c r="G6" s="64" t="inlineStr">
         <is>
           <t>reste (h)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>ACT-01</t>
         </is>
       </c>
-      <c r="B7" s="62" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>Analyse fonctionnelle du besoin</t>
         </is>
       </c>
-      <c r="C7" s="61" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>TERMINEE</t>
         </is>
       </c>
-      <c r="D7" s="61" t="n">
+      <c r="D7" s="65" t="n">
         <v>100</v>
       </c>
-      <c r="E7" s="63" t="n">
+      <c r="E7" s="67" t="n">
         <v>24</v>
       </c>
-      <c r="F7" s="63" t="n">
+      <c r="F7" s="67" t="n">
         <v>22</v>
       </c>
-      <c r="G7" s="63" t="n">
+      <c r="G7" s="67" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="65" t="inlineStr">
         <is>
           <t>ACT-02</t>
         </is>
       </c>
-      <c r="B8" s="62" t="inlineStr">
+      <c r="B8" s="66" t="inlineStr">
         <is>
           <t>Specification des exigences</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="65" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="D8" s="61" t="n">
+      <c r="D8" s="65" t="n">
         <v>60</v>
       </c>
-      <c r="E8" s="63" t="n">
+      <c r="E8" s="67" t="n">
         <v>30</v>
       </c>
-      <c r="F8" s="63" t="n">
+      <c r="F8" s="67" t="n">
         <v>28.5</v>
       </c>
-      <c r="G8" s="63" t="n">
+      <c r="G8" s="67" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="65" t="inlineStr">
         <is>
           <t>ACT-03</t>
         </is>
       </c>
-      <c r="B9" s="62" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>Definition d'architecture</t>
         </is>
       </c>
-      <c r="C9" s="61" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>EN_COURS</t>
         </is>
       </c>
-      <c r="D9" s="61" t="n">
+      <c r="D9" s="65" t="n">
         <v>35</v>
       </c>
-      <c r="E9" s="63" t="n">
+      <c r="E9" s="67" t="n">
         <v>40</v>
       </c>
-      <c r="F9" s="63" t="n">
+      <c r="F9" s="67" t="n">
         <v>12</v>
       </c>
-      <c r="G9" s="63" t="n">
+      <c r="G9" s="67" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="65" t="inlineStr">
         <is>
           <t>ACT-04</t>
         </is>
       </c>
-      <c r="B10" s="62" t="inlineStr">
+      <c r="B10" s="66" t="inlineStr">
         <is>
           <t>Calculs et simulations</t>
         </is>
       </c>
-      <c r="C10" s="61" t="inlineStr">
+      <c r="C10" s="65" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="D10" s="61" t="n">
+      <c r="D10" s="65" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="63" t="n">
+      <c r="E10" s="67" t="n">
         <v>35</v>
       </c>
-      <c r="F10" s="63" t="n">
+      <c r="F10" s="67" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="63" t="n">
+      <c r="G10" s="67" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="65" t="inlineStr">
         <is>
           <t>ACT-05</t>
         </is>
       </c>
-      <c r="B11" s="62" t="inlineStr">
+      <c r="B11" s="66" t="inlineStr">
         <is>
           <t>Revue de conception</t>
         </is>
       </c>
-      <c r="C11" s="61" t="inlineStr">
+      <c r="C11" s="65" t="inlineStr">
         <is>
           <t>A_FAIRE</t>
         </is>
       </c>
-      <c r="D11" s="61" t="n">
+      <c r="D11" s="65" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="63" t="n">
+      <c r="E11" s="67" t="n">
         <v>25</v>
       </c>
-      <c r="F11" s="63" t="n">
+      <c r="F11" s="67" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="63" t="n">
+      <c r="G11" s="67" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="61" t="inlineStr">
+      <c r="A12" s="65" t="inlineStr">
         <is>
           <t>ACT-06</t>
         </is>
       </c>
-      <c r="B12" s="62" t="inlineStr">
+      <c r="B12" s="66" t="inlineStr">
         <is>
           <t>Preparation gate review</t>
         </is>
       </c>
-      <c r="C12" s="61" t="inlineStr">
+      <c r="C12" s="65" t="inlineStr">
         <is>
           <t>STAND_BY</t>
         </is>
       </c>
-      <c r="D12" s="61" t="n">
+      <c r="D12" s="65" t="n">
         <v>10</v>
       </c>
-      <c r="E12" s="63" t="n">
+      <c r="E12" s="67" t="n">
         <v>46</v>
       </c>
-      <c r="F12" s="63" t="n">
+      <c r="F12" s="67" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="63" t="n">
+      <c r="G12" s="67" t="n">
         <v>41.4</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H2:L2"/>
+  <mergeCells count="2">
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">
     <cfRule type="dataBar" priority="1">
@@ -2641,7 +2569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2652,186 +2580,158 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="64" t="n"/>
-      <c r="B1" s="65" t="inlineStr">
+      <c r="A1" s="68" t="n"/>
+      <c r="B1" s="69" t="inlineStr">
         <is>
           <t>UO L09U1 — Préparation et passage des IDR</t>
         </is>
       </c>
-      <c r="C1" s="64" t="n"/>
-      <c r="D1" s="64" t="n"/>
-      <c r="E1" s="64" t="n"/>
-      <c r="F1" s="64" t="n"/>
-      <c r="G1" s="64" t="n"/>
-      <c r="H1" s="64" t="n"/>
-      <c r="I1" s="64" t="n"/>
-      <c r="J1" s="64" t="n"/>
-      <c r="K1" s="66" t="inlineStr">
-        <is>
-          <t>Points ouverts — OIL · J. Dujardin</t>
-        </is>
-      </c>
+      <c r="E1" s="68" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="64" t="n"/>
-      <c r="B2" s="67" t="inlineStr">
-        <is>
-          <t>⚙  CLIMATISATION</t>
-        </is>
-      </c>
-      <c r="G2" s="64" t="n"/>
-      <c r="H2" s="67" t="inlineStr">
-        <is>
-          <t>▣  PROJET DEMO</t>
-        </is>
-      </c>
+      <c r="A2" s="68" t="n"/>
+      <c r="B2" s="70" t="inlineStr">
+        <is>
+          <t>CLIMATISATION  —  PROJET DEMO</t>
+        </is>
+      </c>
+      <c r="E2" s="68" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="64" t="n"/>
-      <c r="B3" s="68">
+      <c r="A3" s="68" t="n"/>
+      <c r="B3" s="71">
         <f>HYPERLINK("#Dashboard!A1","⌂ Dashboard")</f>
         <v/>
       </c>
-      <c r="D3" s="68">
+      <c r="C3" s="71">
         <f>HYPERLINK("#Activites!A1","✎ Activités")</f>
         <v/>
       </c>
-      <c r="F3" s="68">
+      <c r="D3" s="71">
         <f>HYPERLINK("#OIL!A1","⚑ OIL")</f>
         <v/>
       </c>
-      <c r="H3" s="64" t="n"/>
-      <c r="I3" s="64" t="n"/>
-      <c r="J3" s="64" t="n"/>
+      <c r="E3" s="68" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1">
-      <c r="A4" s="64" t="n"/>
-      <c r="B4" s="64" t="n"/>
-      <c r="C4" s="64" t="n"/>
-      <c r="D4" s="64" t="n"/>
-      <c r="E4" s="64" t="n"/>
-      <c r="F4" s="64" t="n"/>
-      <c r="G4" s="64" t="n"/>
-      <c r="H4" s="64" t="n"/>
-      <c r="I4" s="64" t="n"/>
-      <c r="J4" s="64" t="n"/>
+      <c r="A4" s="68" t="n"/>
+      <c r="B4" s="68" t="n"/>
+      <c r="C4" s="68" t="n"/>
+      <c r="D4" s="68" t="n"/>
+      <c r="E4" s="68" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="72" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="72" t="inlineStr">
         <is>
           <t>titre</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="72" t="inlineStr">
         <is>
           <t>en_action</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="72" t="inlineStr">
         <is>
           <t>criticite</t>
         </is>
       </c>
-      <c r="E6" s="60" t="inlineStr">
+      <c r="E6" s="72" t="inlineStr">
         <is>
           <t>statut</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="65" t="inlineStr">
         <is>
           <t>PO-001</t>
         </is>
       </c>
-      <c r="B7" s="62" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>Question expert normes EN 45545</t>
         </is>
       </c>
-      <c r="C7" s="61" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>EXPERT</t>
         </is>
       </c>
-      <c r="D7" s="61" t="inlineStr">
+      <c r="D7" s="65" t="inlineStr">
         <is>
           <t>HAUTE</t>
         </is>
       </c>
-      <c r="E7" s="61" t="inlineStr">
+      <c r="E7" s="65" t="inlineStr">
         <is>
           <t>OUVERT</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="61" t="inlineStr">
+      <c r="A8" s="65" t="inlineStr">
         <is>
           <t>PO-002</t>
         </is>
       </c>
-      <c r="B8" s="62" t="inlineStr">
+      <c r="B8" s="66" t="inlineStr">
         <is>
           <t>Attente retour relecture fournisseur</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="65" t="inlineStr">
         <is>
           <t>FOURNISSEUR</t>
         </is>
       </c>
-      <c r="D8" s="61" t="inlineStr">
+      <c r="D8" s="65" t="inlineStr">
         <is>
           <t>MOYENNE</t>
         </is>
       </c>
-      <c r="E8" s="61" t="inlineStr">
+      <c r="E8" s="65" t="inlineStr">
         <is>
           <t>OUVERT</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="65" t="inlineStr">
         <is>
           <t>PO-003</t>
         </is>
       </c>
-      <c r="B9" s="62" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>Acces outil documentaire obtenu</t>
         </is>
       </c>
-      <c r="C9" s="61" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>SE</t>
         </is>
       </c>
-      <c r="D9" s="61" t="inlineStr">
+      <c r="D9" s="65" t="inlineStr">
         <is>
           <t>BASSE</t>
         </is>
       </c>
-      <c r="E9" s="61" t="inlineStr">
+      <c r="E9" s="65" t="inlineStr">
         <is>
           <t>CLOS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="D3:E3"/>
+  <mergeCells count="2">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D9">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="4">

</xml_diff>